<commit_message>
Fill structured eligibility for every opportunity in the tracking sheet
</commit_message>
<xml_diff>
--- a/docs/OPZY_SOURCE_TRACKING.xlsx
+++ b/docs/OPZY_SOURCE_TRACKING.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:Q24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -482,6 +482,10 @@
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="32" customWidth="1" min="14" max="14"/>
+    <col width="32" customWidth="1" min="15" max="15"/>
+    <col width="32" customWidth="1" min="16" max="16"/>
+    <col width="32" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -550,6 +554,26 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Eligible Countries</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Education Levels</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Fields of Study</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Skills</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -613,6 +637,18 @@
           <t>Real — from original seed.sql</t>
         </is>
       </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>graduate, postgraduate</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -676,6 +712,18 @@
           <t>Real — from original seed.sql</t>
         </is>
       </c>
+      <c r="N3" s="2" t="n"/>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>postgraduate</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>Economics, Finance, Public Health, Education, Engineering, Agriculture, Urban Planning, Social Sciences</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -739,6 +787,18 @@
           <t>Real — from original seed.sql</t>
         </is>
       </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>ECOWAS</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>postgraduate</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="n"/>
+      <c r="Q4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -798,6 +858,10 @@
           <t>Real — from original seed.sql</t>
         </is>
       </c>
+      <c r="N5" s="2" t="n"/>
+      <c r="O5" s="2" t="n"/>
+      <c r="P5" s="2" t="n"/>
+      <c r="Q5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -861,6 +925,26 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>graduate, postgraduate</t>
+        </is>
+      </c>
+      <c r="P6" s="4" t="inlineStr">
+        <is>
+          <t>Computer Science, Computer Engineering, Software Engineering</t>
+        </is>
+      </c>
+      <c r="Q6" s="4" t="inlineStr">
+        <is>
+          <t>Python, Go, SQL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -924,6 +1008,26 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>graduate, postgraduate</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="inlineStr">
+        <is>
+          <t>Mathematics, Statistics, Economics, Computer Science, Engineering, Physics</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>SQL, Excel, Power BI</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -989,6 +1093,22 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>graduate, postgraduate</t>
+        </is>
+      </c>
+      <c r="P8" s="4" t="n"/>
+      <c r="Q8" s="4" t="inlineStr">
+        <is>
+          <t>Customer Service, Writing, Communication</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1052,6 +1172,18 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N9" s="4" t="n"/>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>undergraduate, graduate</t>
+        </is>
+      </c>
+      <c r="P9" s="4" t="n"/>
+      <c r="Q9" s="4" t="inlineStr">
+        <is>
+          <t>Figma, UI Design, UX Research</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1115,6 +1247,22 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N10" s="4" t="n"/>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>undergraduate, postgraduate</t>
+        </is>
+      </c>
+      <c r="P10" s="4" t="inlineStr">
+        <is>
+          <t>Computer Science, Computer Engineering, Software Engineering, Information Technology</t>
+        </is>
+      </c>
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>Python, Java, Data Structures</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1178,6 +1326,26 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>undergraduate</t>
+        </is>
+      </c>
+      <c r="P11" s="4" t="inlineStr">
+        <is>
+          <t>Agriculture, Biology, Statistics</t>
+        </is>
+      </c>
+      <c r="Q11" s="4" t="inlineStr">
+        <is>
+          <t>Data Analysis</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1241,6 +1409,18 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>undergraduate</t>
+        </is>
+      </c>
+      <c r="P12" s="4" t="n"/>
+      <c r="Q12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1304,6 +1484,22 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>graduate</t>
+        </is>
+      </c>
+      <c r="P13" s="4" t="inlineStr">
+        <is>
+          <t>Science, Technology, Engineering, Mathematics, Computer Science, Physics, Chemistry, Biology</t>
+        </is>
+      </c>
+      <c r="Q13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1369,6 +1565,18 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>ECOWAS</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>postgraduate</t>
+        </is>
+      </c>
+      <c r="P14" s="4" t="n"/>
+      <c r="Q14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1432,6 +1640,22 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="n"/>
+      <c r="P15" s="4" t="inlineStr">
+        <is>
+          <t>Computer Science, Software Engineering, Design, Public Policy, Political Science</t>
+        </is>
+      </c>
+      <c r="Q15" s="4" t="inlineStr">
+        <is>
+          <t>Python, JavaScript, Figma, Policy Analysis</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1495,6 +1719,14 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N16" s="4" t="n"/>
+      <c r="O16" s="4" t="n"/>
+      <c r="P16" s="4" t="inlineStr">
+        <is>
+          <t>Environmental Science</t>
+        </is>
+      </c>
+      <c r="Q16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1558,6 +1790,18 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="n"/>
+      <c r="P17" s="4" t="n"/>
+      <c r="Q17" s="4" t="inlineStr">
+        <is>
+          <t>Entrepreneurship</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1623,6 +1867,22 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="n"/>
+      <c r="P18" s="4" t="inlineStr">
+        <is>
+          <t>Fine Arts, Creative Writing, Music, Film</t>
+        </is>
+      </c>
+      <c r="Q18" s="4" t="inlineStr">
+        <is>
+          <t>Writing, Illustration, Photography</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1686,6 +1946,26 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>ECOWAS</t>
+        </is>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>postgraduate</t>
+        </is>
+      </c>
+      <c r="P19" s="4" t="inlineStr">
+        <is>
+          <t>Medicine, Public Health, Pharmacy, Nursing, Biomedical Engineering</t>
+        </is>
+      </c>
+      <c r="Q19" s="4" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1749,6 +2029,14 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N20" s="4" t="n"/>
+      <c r="O20" s="4" t="n"/>
+      <c r="P20" s="4" t="n"/>
+      <c r="Q20" s="4" t="inlineStr">
+        <is>
+          <t>Python, JavaScript, Figma, Product Management</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1812,6 +2100,14 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N21" s="4" t="n"/>
+      <c r="O21" s="4" t="n"/>
+      <c r="P21" s="4" t="n"/>
+      <c r="Q21" s="4" t="inlineStr">
+        <is>
+          <t>Data Analysis, Python</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1875,6 +2171,14 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N22" s="4" t="n"/>
+      <c r="O22" s="4" t="n"/>
+      <c r="P22" s="4" t="n"/>
+      <c r="Q22" s="4" t="inlineStr">
+        <is>
+          <t>Entrepreneurship, Public Speaking</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1940,6 +2244,22 @@
           <t>DUMMY — fictional, dev/testing only</t>
         </is>
       </c>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>secondary, undergraduate</t>
+        </is>
+      </c>
+      <c r="P23" s="4" t="n"/>
+      <c r="Q23" s="4" t="inlineStr">
+        <is>
+          <t>Writing</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -2001,6 +2321,26 @@
       <c r="M24" s="4" t="inlineStr">
         <is>
           <t>DUMMY — fictional, dev/testing only</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="O24" s="4" t="inlineStr">
+        <is>
+          <t>undergraduate</t>
+        </is>
+      </c>
+      <c r="P24" s="4" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="Q24" s="4" t="inlineStr">
+        <is>
+          <t>Python, Java</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2135,40 +2475,88 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Eligible Countries</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Comma-separated ISO codes (NG, GH, …) or ECOWAS. Blank = any country. Hard filter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Education Levels</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Comma-separated: secondary, undergraduate, graduate (first degree/HND, not studying), postgraduate. Blank = any level. Hard filter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Fields of Study</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Comma-separated fields it wants, e.g. Computer Science. Blank = any. Ranking only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Skills</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Comma-separated skills it asks for, e.g. Python, SQL. Blank = none listed. Ranking only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Not imported. Rows marked DUMMY (shaded) are fictional test data — replace before launch.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-      <c r="B11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>To add an opportunity</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Add a new row on the Opportunities tab, copying the format of row 2.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Generated</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>2026-09-18 — 4 real rows (from seed.sql) + 19 dummy rows</t>
         </is>

</xml_diff>